<commit_message>
output files from troubleshooting on Sept 17 to clean up cash
</commit_message>
<xml_diff>
--- a/4.1 Myrmidon Happy reef/output/Rugosity_growth_param_0.5.xlsx
+++ b/4.1 Myrmidon Happy reef/output/Rugosity_growth_param_0.5.xlsx
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.386432714524236</v>
+        <v>1.402004812151946</v>
       </c>
     </row>
     <row r="4">
@@ -456,7 +456,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.381000966139834</v>
+        <v>1.413508780798003</v>
       </c>
     </row>
     <row r="5">
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.375442752424855</v>
+        <v>1.422646911946286</v>
       </c>
     </row>
     <row r="6">
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.384974732817064</v>
+        <v>1.459705697956153</v>
       </c>
     </row>
     <row r="7">
@@ -480,7 +480,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1.396321521455336</v>
+        <v>1.495798473321962</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1.425643253001748</v>
+        <v>1.550374452454609</v>
       </c>
     </row>
     <row r="9">
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1.476633349695222</v>
+        <v>1.627514059229768</v>
       </c>
     </row>
     <row r="10">
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.544720063313617</v>
+        <v>1.716354411570539</v>
       </c>
     </row>
     <row r="11">
@@ -512,7 +512,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1.632648037933889</v>
+        <v>1.816705877450247</v>
       </c>
     </row>
     <row r="12">
@@ -520,7 +520,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1.745355904822244</v>
+        <v>1.932781588688277</v>
       </c>
     </row>
     <row r="13">
@@ -528,7 +528,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>1.957218900175651</v>
+        <v>2.080946506243148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
follow up to the previous commit to push all the changed files
</commit_message>
<xml_diff>
--- a/4.1 Myrmidon Happy reef/output/Rugosity_growth_param_0.5.xlsx
+++ b/4.1 Myrmidon Happy reef/output/Rugosity_growth_param_0.5.xlsx
@@ -448,7 +448,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1.402004812151946</v>
+        <v>1.399997999559417</v>
       </c>
     </row>
     <row r="4">
@@ -456,7 +456,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1.413508780798003</v>
+        <v>1.409254081687253</v>
       </c>
     </row>
     <row r="5">
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1.422646911946286</v>
+        <v>1.416495017004452</v>
       </c>
     </row>
     <row r="6">
@@ -472,7 +472,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1.459705697956153</v>
+        <v>1.450208211215427</v>
       </c>
     </row>
     <row r="7">
@@ -480,7 +480,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>1.495798473321962</v>
+        <v>1.48371015577396</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1.550374452454609</v>
+        <v>1.535257592075599</v>
       </c>
     </row>
     <row r="9">
@@ -496,7 +496,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>1.627514059229768</v>
+        <v>1.608528393009339</v>
       </c>
     </row>
     <row r="10">
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>1.716354411570539</v>
+        <v>1.694031343842311</v>
       </c>
     </row>
     <row r="11">
@@ -512,7 +512,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>1.816705877450247</v>
+        <v>1.791889345277475</v>
       </c>
     </row>
     <row r="12">
@@ -520,7 +520,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>1.932781588688277</v>
+        <v>1.907568366481611</v>
       </c>
     </row>
     <row r="13">
@@ -528,7 +528,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>2.080946506243148</v>
+        <v>2.055169584748539</v>
       </c>
     </row>
   </sheetData>

</xml_diff>